<commit_message>
feat: implement multi-agent architecture with SQL, graph, and RAG agents alongside MCP server integration
</commit_message>
<xml_diff>
--- a/benchmark/benchmark2.xlsx
+++ b/benchmark/benchmark2.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alejandro\DATAX\TrabajoDirigido\Analyst_DATAX\benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4DC323B-5D66-4ACB-B5CC-EEC72E1AF06A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5ED0987-D073-4158-82E8-39BC2F63916D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-132" yWindow="-132" windowWidth="41544" windowHeight="16824" activeTab="1" xr2:uid="{C5EA59B6-CBD3-49E2-BAF7-A3DA1019A7B6}"/>
+    <workbookView xWindow="-132" yWindow="-132" windowWidth="41544" windowHeight="16824" activeTab="3" xr2:uid="{C5EA59B6-CBD3-49E2-BAF7-A3DA1019A7B6}"/>
   </bookViews>
   <sheets>
     <sheet name="benchmark - Hoja 1" sheetId="2" r:id="rId1"/>
     <sheet name="Hoja_grafos" sheetId="1" r:id="rId2"/>
-    <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja_grafos2" sheetId="3" r:id="rId3"/>
+    <sheet name="Hoja_grafos3" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="0" hidden="1">'benchmark - Hoja 1'!$A$1:$M$11</definedName>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="164">
   <si>
     <t>Column1</t>
   </si>
@@ -872,6 +873,535 @@
     <t>EL banco de crédito (BCR) seguramente tiene un spread con el que opera la intermediación de depósitos y la colocación de créditos en cartera. Ese spread tiene que cubrir gastos por incobrabilidad, gastos administrativos, costo de los fondos que usa y demás.
 Lo que necesito saber es cuánto es el costo de los fondos de este banco en estas últimas 2 gestiones (2024, 2025) que deberia ser considerado para saber cuánto consume ese gastos del spread efectivo del banco.
 Te pongo un ejemplo: Si se calcula que el spread del banco es de 7 (es decir 7% o 7 puntos porcentuales) y se sabe que el costo de los fondos es de 2.5 (2.5% o 2.5 puntos porcentuales), sabría que le sobran 4.5 puntos para cubrir gastos de impagos, gastos administrativos y otros para finalizar conociendo el porcentaje destinado del spread a la utilidad. Lo que necesito saber es ese porcentaje del costo de fondos (en el ejemplo 2.5%) de las gestiones 2024 y 2025.</t>
+  </si>
+  <si>
+    <t>pregunta</t>
+  </si>
+  <si>
+    <t>respuesta esperada</t>
+  </si>
+  <si>
+    <t>intento1</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Saldo Bs") AS "monto_activo_disponible_bs" 
+FROM "S_BOSBEF44_000392" 
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3 
+AND "Mes" = 'Diciembre' 
+AND "Entidad Financiera" = 'BIS' 
+AND "Cuenta Nv1" = '100.00 ACTIVO' 
+AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES' 
+GROUP BY "Año" 
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Saldo Bs") AS "monto_activo_disponible_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Tipo Entidad Financiera" IN ('Banco', 'Banco Múltiple')
+  AND "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Saldo Bs") AS "monto_disponibilidades_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Entidad Financiera" = 'BIS'
+  AND (
+    "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+    OR "Cuenta Nv3" IN ('871.00 DISPONIBILIDADES', '881.00 DISPONIBILIDADES')
+  )
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>Lamentablemente, no se ha encontrado información existente en la base de datos sobre el monto del activo disponible con el que cerró su gestión BISA seguros en los últimos 3 años.
+Esto podría deberse a la falta de tablas específicas que contengan conceptos equivalentes a activo disponible o disponibilidades al cierre de gestión para esa entidad en particular.
+Si tienes más preguntas o alguna otra consulta, estaré encantado de ayudarte.</t>
+  </si>
+  <si>
+    <t>Lamentablemente, no se encontraron datos específicos relacionados con el monto del activo disponible con el que cerró su gestión "BISA Seguros" en los últimos 3 años. Esto podría deberse a la falta de información precisa en las tablas relacionadas con seguros o el cierre de gestión.
+Si puedes proporcionar más detalles o enfoques alternativos, estaré encantado de intentar ayudar nuevamente.</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "monto_disponible_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv4" IN ('425020101 Disponible', '425030101 Disponible', '425010101 Disponible', '525030201 Disponible')
+  AND "Mes" = 'Diciembre'
+  AND "Año" IN (
+    SELECT DISTINCT "Año"
+    FROM "S_BOAPS_44_000612"
+    ORDER BY "Año" DESC
+    LIMIT 3
+  )
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Saldo Bs") AS monto_disponible_bs
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";
+SELECT "Año", SUM("Monto Acumulado Bs") AS monto_disponible_bs
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>intento2</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS monto_disponible_bs
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "monto_depositado_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv4" IN (
+    '1010201 Bancos',
+    '523040301 Bancos del país',
+    '523050201 Bancos comerciales nacionales',
+    '523050202 Bancos comerciales extranjeros',
+    '422020101 Bancos comerciales nacionales',
+    '422020201 Bancos comerciales nacionales',
+    '1070301 Depósitos Judiciales'
+  )
+  AND "Aseguradora" = 'BISA'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT 
+  "Año", 
+  SUM("Monto Acumulado Bs") AS "monto_bs_depositado_en_bancos" 
+FROM 
+  "S_BOAPS_44_000612" 
+WHERE 
+  "Aseguradora" = 'BISA' 
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
+  AND "Mes" = 'Diciembre' 
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE' 
+  AND (
+    "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS' 
+    OR "Cuenta Financiera Nv4" IN ('523040301 Bancos del país', '523040302 Bancos del exterior', '523050201 Bancos comerciales nacionales', '523050202 Bancos comerciales extranjeros')
+  ) 
+GROUP BY 
+  "Año" 
+ORDER BY 
+  "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  c."Año",
+  c."Trimestre",
+  c.cartera_vencida_consumo_bs,
+  g.cartera_garantia_depositos_bs,
+  CASE
+    WHEN g.cartera_garantia_depositos_bs = 0 THEN NULL
+    ELSE c.cartera_vencida_consumo_bs / g.cartera_garantia_depositos_bs
+  END AS proporcion_vencida_sobre_garantia
+FROM (
+  SELECT
+    "Año",
+    "Trimestre",
+    SUM("Monto Bs") AS cartera_vencida_consumo_bs
+  FROM "S_BOASFI66_000728"
+  WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+    AND "Trimestre" = 'IV'
+    AND "Entidad" = 'BNA'
+    AND "Estado Cartera" = 'Vencida'
+    AND "Tipo Crédito" IN ('Crédito de Consumo', 'Crédito de Consumo debidamente Garantizado')
+  GROUP BY "Año", "Trimestre"
+) c
+CROSS JOIN (
+  SELECT
+    SUM("Monto Bs") AS cartera_garantia_depositos_bs
+  FROM "clf_crt_tip_gar"
+  WHERE "Año" = (SELECT MAX("Año") FROM "clf_crt_tip_gar")
+    AND "Trimestre" = 'IV'
+    AND "Entidad" = 'BNA'
+    AND "Garantía Nv1" = 'Depositos en la Entidad Financiera'
+) g;</t>
+  </si>
+  <si>
+    <t>No existe la informacion</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Bs") AS "cartera_vencida_bs"
+FROM "S_BOASFI66_000728"
+WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+  AND "Trimestre" = 'IV'
+  AND "Entidad" = 'BNA'
+  AND "Estado Cartera" = 'Vencida'
+  AND "Tipo Crédito" = 'Crédito de Consumo debidamente Garantizado'
+GROUP BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", "Entidad Financiera", "Indicador Nv2", "Indicador %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+AND "Mes" = 'Diciembre'
+AND "Año" &gt;= (SELECT MAX("Año") FROM "SPIM_50013_IF") - 1
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT "Año", "Indicador %" AS "Costo de los fondos"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+AND "Mes" = 'diciembre'
+AND "Año" &gt;= (SELECT MAX("Año") FROM "SPIM_50013_IF") - 1
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT 
+  "Año", 
+  MAX(CASE WHEN "Indicador Nv2" = 'UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO' THEN "Indicador %" END) AS "utilizacion_spread_efectivo_spread_efectivo", 
+  MAX(CASE WHEN "Indicador Nv2" = 'CÁLCULO SPREAD EFECTIVO - SPREAD EFECTIVO' THEN "Indicador %" END) AS "calculo_spread_efectivo_spread_efectivo" 
+FROM "S_BOFINR44_00387" 
+WHERE 
+  "Entidad Financiera" = 'Banco de Crédito' 
+  AND "Indicador Nv2" IN ('UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO', 'CÁLCULO SPREAD EFECTIVO - SPREAD EFECTIVO') 
+  AND "Año" &gt;= (SELECT MAX("Año") FROM "S_BOFINR44_00387") - 2 
+  AND "Año" &lt; (SELECT MAX("Año") FROM "S_BOFINR44_00387") 
+  AND "Mes" = 'diciembre' 
+GROUP BY "Año" 
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT 
+    "Año", 
+    AVG(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END) AS "spread_efectivo_promedio", 
+    AVG(CASE WHEN "Indicador Nv2" = 'Costo Promedio de Fondos' THEN "Indicador %" END) AS "costo_promedio_fondos_promedio", 
+    AVG(CASE WHEN "Indicador Nv2" = 'Costo Promedio de Fondos' THEN "Indicador %" END) / NULLIF(AVG(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END), 0) AS "proporcion_costo_sobre_spread" 
+FROM "SPIM_50013_IF" 
+WHERE "Entidad Financiera" = 'BCR' 
+AND "Indicador Nv2" IN ('SPREAD EFECTIVO', 'Costo Promedio de Fondos') 
+AND "Año" &gt;= (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2 
+AND "Año" &lt; (SELECT MAX("Año") FROM "SPIM_50013_IF") 
+GROUP BY "Año" 
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>EL banco de crédito (BCR) seguramente tiene un spread con el que opera la intermediación de depósitos y la colocación de créditos en cartera. Ese spread tiene que cubrir gastos por incobrabilidad, gastos administrativos, costo de los fondos que usa y demás. Lo que necesito saber es cuánto es el costo de los fondos de este banco en estas últimas 2 gestiones (2024, 2025) que deberia ser considerado para saber cuánto consume ese gastos del spread efectivo del banco. Te pongo un ejemplo: Si se calcula que el spread del banco es de 7 (es decir 7% o 7 puntos porcentuales) y se sabe que el costo de los fondos es de 2.5 (2.5% o 2.5 puntos porcentuales), sabría que le sobran 4.5 puntos para cubrir gastos de impagos, gastos administrativos y otros para finalizar conociendo el porcentaje destinado del spread a la utilidad. Lo que necesito saber es ese porcentaje del costo de fondos (en el ejemplo 2.5%) de las gestiones 2024 y 2025.</t>
+  </si>
+  <si>
+    <t>SELECT "Año", AVG("Indicador %") AS "costo_promedio_fondos"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+AND "Indicador Nv2" = 'Costo Promedio de Fondos'
+AND "Año" IN (2024, 2025)
+AND "Mes" = 'diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", "Mes", "Entidad Financiera", "Tipo Entidad", "Indicador Nv1", "Indicador Nv2", "Indicador %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Año" IN (2024, 2025)
+  AND "Tipo Entidad" = 'Banco'
+  AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+ORDER BY "Año", "Mes";</t>
+  </si>
+  <si>
+    <t>intento3</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Entidad Financiera" = 'BIS'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Saldo Bs" AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Entidad Financiera" = 'BIS'
+  AND "Tipo Entidad Financiera" = 'Banco'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Saldo Bs") AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "Monto_Activo_Disponible_Bs" 
+FROM "S_BOAPS_44_000612" 
+WHERE "Aseguradora" = 'BISA' 
+AND "Cuenta Financiera Nv1" = '1 ACTIVO' 
+AND "Cuenta Financiera Nv2" = '101 DISPONIBLE' 
+AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+AND "Mes" = 'Diciembre' 
+AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
+GROUP BY "Año" ORDER BY "Año" DESC;v</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "Monto_Activo_Disponible_Bs" 
+FROM "S_BOAPS_44_000612" 
+WHERE "Aseguradora" = 'BISA' 
+AND "Cuenta Financiera Nv1" = '1 ACTIVO' 
+AND "Cuenta Financiera Nv2" = '101 DISPONIBLE' 
+AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+AND "Mes" = 'Diciembre' 
+AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
+GROUP BY "Año" ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_disponible_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_depositado_en_bancos_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv4" = 'Bancos comerciales nacionales/extranjeros'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_depositado_en_bancos_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND "Cuenta Financiera Nv4" IN ('Bancos comerciales nacionales', 'Bancos comerciales extranjeros')
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de los fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Tipo Entidad" = 'Banco'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  c."Año",
+  SUM(c."Monto Bs") AS "cartera_vencida_consumo_bs"
+FROM "S_BOASFI66_000728" c
+WHERE c."Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+  AND c."Trimestre" = 'IV'
+  AND c."Tipo Crédito" = 'Crédito de Consumo'
+  AND c."Estado Cartera" = 'Vencida'
+  AND c."Entidad" = 'BNA'
+  AND c."Tipo Entidad" IN ('Banco Múltiple', 'Banco PyME')
+  AND EXISTS (
+    SELECT 1
+    FROM "clf_crt_tip_gar" g
+    WHERE g."Año" = c."Año"
+      AND g."Trimestre" = c."Trimestre"
+      AND g."Entidad" = c."Entidad"
+      AND g."Tipo Entidad" = c."Tipo Entidad"
+      AND g."Garantía Nv1" = 'Depositos en la Entidad Financiera'
+  )
+GROUP BY c."Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  c."Año",
+  c."Trimestre",
+  c."Monto Bs" AS "cartera_vencida_bs"
+FROM "S_BOASFI66_000728" c
+INNER JOIN "clf_crt_tip_gar" g
+  ON c."Año" = g."Año"
+ AND c."Trimestre" = g."Trimestre"
+ AND c."Entidad" = g."Entidad"
+WHERE c."Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+  AND c."Trimestre" = 'IV'
+  AND c."Entidad" = 'BNA'
+  AND c."Tipo Crédito" = 'Crédito de Consumo'
+  AND c."Estado Cartera" = 'Vencida'
+  AND g."Garantía Nv1" = 'Depositos en la Entidad Financiera';</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG(CASE
+        WHEN "Indicador Nv1" = 'UTILIZACIÓN DEL SPREAD EFECTIVO'
+         AND "Indicador Nv2" = 'Costo Promedio de Fondos'
+        THEN "Indicador %"
+      END) AS "porcentaje_spread_usado_para_cubrir_costo_fondos"
+FROM "S_BOFINR44_00387"
+WHERE "Entidad Financiera" = 'BANCO DE CRÉDITO'
+  AND "Año" &gt;= (SELECT MAX("Año") FROM "S_BOFINR44_00387") - 1
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END) AS "spread_efectivo",
+  MAX(CASE WHEN "Indicador Nv2" = 'Costo Promedio de Fondos' THEN "Indicador %" END) AS "costo_promedio_fondos",
+  CASE
+    WHEN MAX(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END) = 0 THEN NULL
+    ELSE MAX(CASE WHEN "Indicador Nv2" = 'Costo Promedio de Fondos' THEN "Indicador %" END)
+         / MAX(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END)
+  END AS "proporcion_del_spread_usada_para_cubrir_costo_fondos"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" IN ('SPREAD EFECTIVO', 'Costo Promedio de Fondos')
+  AND "Año" &gt;= (SELECT MAX("Año") FROM "SPIM_50013_IF") - 1
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT "Año", AVG("Indicador %") AS "Costo Promedio de Fondos"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Indicador %") AS "Costo Promedio de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
   </si>
 </sst>
 </file>
@@ -1947,9 +2477,309 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F382CB-3264-4364-8BC0-86B6B1186798}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72D89B5-A94F-4B95-9307-F1034D484F2C}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: implementation of 'Intent-Depth Mapping' and 'Pure Transmission' architecture for multi-agent RAG pipeline
</commit_message>
<xml_diff>
--- a/benchmark/benchmark2.xlsx
+++ b/benchmark/benchmark2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alejandro\DATAX\TrabajoDirigido\Analyst_DATAX\benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5ED0987-D073-4158-82E8-39BC2F63916D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7369DCBE-D2DD-41C9-A2E6-6351078409B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-132" yWindow="-132" windowWidth="41544" windowHeight="16824" activeTab="3" xr2:uid="{C5EA59B6-CBD3-49E2-BAF7-A3DA1019A7B6}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="185">
   <si>
     <t>Column1</t>
   </si>
@@ -1211,17 +1211,6 @@
 AND "Cuenta Financiera Nv4" = '1010201 Bancos'
 AND "Mes" = 'Diciembre' 
 AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
-GROUP BY "Año" ORDER BY "Año" DESC;v</t>
-  </si>
-  <si>
-    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "Monto_Activo_Disponible_Bs" 
-FROM "S_BOAPS_44_000612" 
-WHERE "Aseguradora" = 'BISA' 
-AND "Cuenta Financiera Nv1" = '1 ACTIVO' 
-AND "Cuenta Financiera Nv2" = '101 DISPONIBLE' 
-AND "Cuenta Financiera Nv4" = '1010201 Bancos'
-AND "Mes" = 'Diciembre' 
-AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
 GROUP BY "Año" ORDER BY "Año" DESC;</t>
   </si>
   <si>
@@ -1401,6 +1390,332 @@
   AND "Año" IN (2024, 2025)
   AND "Mes" = 'Diciembre'
 GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>intento4</t>
+  </si>
+  <si>
+    <t>intento5</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto") AS "monto_activo_disponible"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "activo_disponible_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Cuenta Nv2",
+  "Saldo Bs" AS "monto_disponibilidades_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto") AS "monto_disponibilidades"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", SUM("Monto Acumulado Bs") AS "Monto_Activo_Disponible_Bs" 
+FROM "S_BOAPS_44_000612" 
+WHERE "Aseguradora" = 'BISA' 
+AND "Cuenta Financiera Nv1" = '1 ACTIVO' 
+AND "Cuenta Financiera Nv2" = '101 DISPONIBLE' 
+AND "Mes" = 'Diciembre' 
+AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3 
+GROUP BY "Año" ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "Activo Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Aseguradora",
+  "Cuenta Financiera Nv4",
+  "Monto Acumulado Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv4" = '422020101 Bancos comerciales nacionales'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "Monto Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "Monto depositado en bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv5" = '103030101 Bancos del país'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_depositado_bancos_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>WITH cartera_consumo_total AS (
+    SELECT
+        "Año",
+        SUM("Monto Bs") AS total_consumo_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+      AND "Entidad" = 'BNA'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+    GROUP BY "Año"
+),
+cartera_consumo_vencida AS (
+    SELECT
+        "Año",
+        SUM("Monto Bs") AS vencida_consumo_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+      AND "Entidad" = 'BNA'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+      AND "Estado Cartera" = 'Vencida'
+    GROUP BY "Año"
+)
+SELECT
+    t."Año",
+    t.total_consumo_bs,
+    v.vencida_consumo_bs,
+    CASE
+        WHEN t.total_consumo_bs = 0 THEN NULL
+        ELSE v.vencida_consumo_bs / t.total_consumo_bs
+    END AS ratio_vencida_sobre_total
+FROM cartera_consumo_total t
+LEFT JOIN cartera_consumo_vencida v
+    ON t."Año" = v."Año";</t>
+  </si>
+  <si>
+    <t>WITH cartera_consumo_total AS (
+    SELECT
+        "Año",
+        "Trimestre",
+        SUM("Monto Bs") AS total_cartera_consumo_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Entidad" = 'BNA'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+      AND "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+    GROUP BY "Año", "Trimestre"
+),
+cartera_consumo_vencida AS (
+    SELECT
+        "Año",
+        "Trimestre",
+        SUM("Monto Bs") AS cartera_vencida_consumo_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Entidad" = 'BNA'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+      AND "Estado Cartera" = 'Vencida'
+      AND "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+    GROUP BY "Año", "Trimestre"
+),
+cartera_con_garantia_depositos AS (
+    SELECT
+        "Año",
+        "Trimestre",
+        SUM("Monto Bs") AS cartera_garantia_depositos_bs
+    FROM "clf_crt_tip_gar"
+    WHERE "Entidad" = 'BNA'
+      AND "Garantía Nv1" = 'Depositos en la Entidad Financiera'
+      AND "Año" = (SELECT MAX("Año") FROM "clf_crt_tip_gar")
+      AND "Trimestre" = 'IV'
+    GROUP BY "Año", "Trimestre"
+)
+SELECT
+    t."Año",
+    t."Trimestre",
+    t.total_cartera_consumo_bs,
+    v.cartera_vencida_consumo_bs,
+    g.cartera_garantia_depositos_bs
+FROM cartera_consumo_total t
+LEFT JOIN cartera_consumo_vencida v
+    ON t."Año" = v."Año"
+   AND t."Trimestre" = v."Trimestre"
+LEFT JOIN cartera_con_garantia_depositos g
+    ON t."Año" = g."Año"
+   AND t."Trimestre" = g."Trimestre";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de los Fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de los fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  se."Año",
+  se."Entidad Financiera",
+  se."Indicador %" AS "Spread Efectivo",
+  cf."Indicador %" AS "Costo Promedio de Fondos",
+  CASE
+    WHEN se."Indicador %" &lt;&gt; 0 THEN cf."Indicador %" / se."Indicador %"
+    ELSE NULL
+  END AS "Proporcion del spread usada para cubrir costo de fondos"
+FROM "SPIM_50013_IF" se
+JOIN "SPIM_50013_IF" cf
+  ON se."Año" = cf."Año"
+ AND se."Mes" = cf."Mes"
+ AND se."Entidad Financiera" = cf."Entidad Financiera"
+WHERE se."Entidad Financiera" = 'BCR'
+  AND se."Indicador Nv2" = 'SPREAD EFECTIVO'
+  AND cf."Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND se."Año" &gt;= (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND se."Año" &lt; (SELECT MAX("Año") FROM "SPIM_50013_IF")
+  AND se."Mes" = 'Diciembre'
+  AND cf."Mes" = 'Diciembre'
+ORDER BY se."Año";</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>SELECT
+  t."Año",
+  t."Entidad Financiera",
+  MAX(CASE WHEN t."Indicador Nv2" = 'UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO' THEN t."Indicador %" END) AS "Spread Efectivo %",
+  MAX(CASE WHEN t."Indicador Nv2" = 'Costo Promedio de Fondos' THEN t."Indicador %" END) AS "Costo de Fondos %",
+  CASE
+    WHEN MAX(CASE WHEN t."Indicador Nv2" = 'UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO' THEN t."Indicador %" END) = 0 THEN NULL
+    ELSE
+      MAX(CASE WHEN t."Indicador Nv2" = 'Costo Promedio de Fondos' THEN t."Indicador %" END)
+      / MAX(CASE WHEN t."Indicador Nv2" = 'UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO' THEN t."Indicador %" END)
+    END AS "Proporcion del spread usada para cubrir costo de fondos"
+FROM "S_BOFINR44_00387" t
+WHERE t."Año" &gt;= (SELECT MAX("Año") FROM "S_BOFINR44_00387") - 2
+  AND t."Año" &lt; (SELECT MAX("Año") FROM "S_BOFINR44_00387")
+  AND t."Mes" = 'Diciembre'
+  AND t."Indicador Nv2" IN (
+    'UTILIZACIÓN DEL SPREAD EFECTIVO - SPREAD EFECTIVO',
+    'Costo Promedio de Fondos'
+  )
+GROUP BY t."Año", t."Entidad Financiera"
+ORDER BY t."Año", t."Entidad Financiera";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Indicador %" AS "Costo de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Tipo Entidad" = 'Banco Múltiple'
+  AND "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Indicador %" AS "Costo de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
 ORDER BY "Año";</t>
   </si>
 </sst>
@@ -1425,12 +1740,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1445,12 +1766,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2624,10 +2946,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72D89B5-A94F-4B95-9307-F1034D484F2C}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -2643,8 +2965,14 @@
       <c r="E1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F1" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2660,8 +2988,14 @@
       <c r="E2" s="1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F2" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -2677,39 +3011,57 @@
       <c r="E3" s="1" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F3" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>96</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>149</v>
+        <v>169</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+        <v>150</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>106</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F5" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>108</v>
       </c>
@@ -2717,13 +3069,19 @@
         <v>129</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F6" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -2731,13 +3089,19 @@
         <v>133</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F7" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -2745,27 +3109,39 @@
         <v>116</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F8" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>181</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>116</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="F9" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -2773,10 +3149,16 @@
         <v>116</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>163</v>
+      <c r="F10" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement hierarchical lineage and deterministic SQL path suggestions
</commit_message>
<xml_diff>
--- a/benchmark/benchmark2.xlsx
+++ b/benchmark/benchmark2.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alejandro\DATAX\TrabajoDirigido\Analyst_DATAX\benchmark\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7369DCBE-D2DD-41C9-A2E6-6351078409B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD0B24EC-39F4-451C-BBEA-D8D133259A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-132" yWindow="-132" windowWidth="41544" windowHeight="16824" activeTab="3" xr2:uid="{C5EA59B6-CBD3-49E2-BAF7-A3DA1019A7B6}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{C5EA59B6-CBD3-49E2-BAF7-A3DA1019A7B6}"/>
   </bookViews>
   <sheets>
     <sheet name="benchmark - Hoja 1" sheetId="2" r:id="rId1"/>
     <sheet name="Hoja_grafos" sheetId="1" r:id="rId2"/>
     <sheet name="Hoja_grafos2" sheetId="3" r:id="rId3"/>
     <sheet name="Hoja_grafos3" sheetId="4" r:id="rId4"/>
+    <sheet name="Hoja_grafos4" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="DatosExternos_1" localSheetId="0" hidden="1">'benchmark - Hoja 1'!$A$1:$M$11</definedName>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="227">
   <si>
     <t>Column1</t>
   </si>
@@ -1718,6 +1719,743 @@
   AND "Mes" = 'Diciembre'
 ORDER BY "Año";</t>
   </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "monto_activo_disponible_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "order Cuenta Nv3" = '11'
+  AND "Cuenta Nv3" = '113.00 BANCOS Y CORRESPONSALES DEL PAÍS'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Saldo Bs" AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "order Cuenta Nv2" = 1
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "orden Cuenta Financiera Nv1" = 1
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "orden Cuenta Financiera Nv2" = 10
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Aseguradora" = 'BISA'
+  AND "orden Cuenta Financiera Nv1" = '1'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "orden Cuenta Financiera Nv2" = '10'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_depositado_en_bancos_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND (
+    ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '103050101 Bancos comerciales nacionales')
+    OR ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '104010201 Bancos comerciales nacionales')
+    OR ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '104890201 Bancos comerciales nacionales')
+    OR ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '106010201 Bancos comerciales nacionales')
+    OR ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '103030101 Bancos del país')
+    OR ("orden Cuenta Financiera Nv5" = '10' AND "Cuenta Financiera Nv5" = '103890301 Bancos del país')
+  )
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de los fondos"
+FROM "S_BOFINR44_00387"
+WHERE "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOFINR44_00387") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>WITH cartera_consumo_total AS (
+    SELECT SUM("Monto Bs") AS total_monto_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+      AND "Entidad" = 'BNA'
+      AND "Tipo Entidad" = 'Banco Múltiple'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+),
+cartera_vencida_consumo AS (
+    SELECT SUM("Monto Bs") AS vencida_monto_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+      AND "Trimestre" = 'IV'
+      AND "Entidad" = 'BNA'
+      AND "Tipo Entidad" = 'Banco Múltiple'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+      AND "Estado Cartera" = 'Vencida'
+)
+SELECT 
+    t.total_monto_bs AS "Cartera total consumo Bs",
+    v.vencida_monto_bs AS "Cartera vencida consumo Bs",
+    CASE 
+        WHEN t.total_monto_bs &gt; 0 THEN v.vencida_monto_bs / t.total_monto_bs
+        ELSE NULL
+    END AS "Proporcion vencida sobre total"
+FROM cartera_consumo_total t
+CROSS JOIN cartera_vencida_consumo v;</t>
+  </si>
+  <si>
+    <t>SELECT
+  se."Año",
+  MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END) AS "spread_efectivo_pct",
+  MAX(CASE WHEN se."Indicador Nv2" = '   Costo Promedio de Fondos' THEN se."Indicador %" END) AS "costo_promedio_fondos_pct",
+  CASE
+    WHEN MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END) = 0 THEN NULL
+    ELSE MAX(CASE WHEN se."Indicador Nv2" = '   Costo Promedio de Fondos' THEN se."Indicador %" END)
+         / MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END)
+  END AS "proporcion_del_spread_destinada_a_cubrir_costo_fondos"
+FROM "SPIM_50013_IF" se
+WHERE se."Indicador Nv2" IN ('SPREAD EFECTIVO', '   Costo Promedio de Fondos')
+  AND se."Entidad Financiera" = 'BCR'
+  AND se."Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND se."Mes" = 'Diciembre'
+GROUP BY se."Año"
+ORDER BY se."Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Mes",
+  "Indicador %" AS "Costo de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+ORDER BY "Año", "Mes";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "monto_activo_disponible_bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv1" = '100.00 ACTIVO'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Activo Disponible Cierre Gestion Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "monto_disponible_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto depositado en bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  c."Año",
+  c."Trimestre",
+  c."Entidad",
+  SUM(CASE WHEN c."Estado Cartera" = 'Vencida' THEN c."Monto Bs" ELSE 0 END) AS "cartera_vencida_consumo_bs",
+  SUM(c."Monto Bs") AS "cartera_total_consumo_bs",
+  CASE
+    WHEN SUM(c."Monto Bs") = 0 THEN NULL
+    ELSE SUM(CASE WHEN c."Estado Cartera" = 'Vencida' THEN c."Monto Bs" ELSE 0 END) / SUM(c."Monto Bs")
+  END AS "ratio_cartera_vencida"
+FROM "S_BOASFI66_000728" c
+WHERE c."Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+  AND c."Trimestre" = 'IV'
+  AND c."Entidad" = 'BNA'
+  AND c."Tipo Crédito" = 'Crédito de Consumo'
+GROUP BY c."Año", c."Trimestre", c."Entidad";
+SELECT
+  g."Año",
+  g."Trimestre",
+  g."Entidad",
+  SUM(g."Monto Bs") AS "cartera_bs_garantia_depositos_entidad"
+FROM "clf_crt_tip_gar" g
+WHERE g."Año" = (SELECT MAX("Año") FROM "clf_crt_tip_gar")
+  AND g."Trimestre" = 'IV'
+  AND g."Entidad" = 'BNA'
+  AND g."Garantía Nv1" = 'Depositos en la Entidad Financiera'
+GROUP BY g."Año", g."Trimestre", g."Entidad";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "costo_fondos"
+FROM "S_BOFINR44_00387"
+WHERE "Indicador Nv2" = 'Costo Promedio de Fondos'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOFINR44_00387") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>WITH max_anio AS (
+    SELECT MAX("Año") AS anio_max
+    FROM "SPIM_50013_IF"
+),
+spread AS (
+    SELECT
+        "Año",
+        AVG("Indicador %") AS spread_efectivo
+    FROM "SPIM_50013_IF"
+    WHERE "Año" &gt; (SELECT anio_max FROM max_anio) - 2
+      AND "Mes" = 'Diciembre'
+      AND "Entidad Financiera" = 'BCR'
+      AND "Tipo Entidad" = 'Banco'
+      AND "Indicador Nv2" = 'SPREAD EFECTIVO'
+    GROUP BY "Año"
+),
+costo AS (
+    SELECT
+        "Año",
+        AVG("Indicador %") AS costo_fondos
+    FROM "SPIM_50013_IF"
+    WHERE "Año" &gt; (SELECT anio_max FROM max_anio) - 2
+      AND "Mes" = 'Diciembre'
+      AND "Entidad Financiera" = 'BCR'
+      AND "Tipo Entidad" = 'Banco'
+      AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+    GROUP BY "Año"
+)
+SELECT
+    s."Año",
+    s.spread_efectivo,
+    c.costo_fondos,
+    CASE
+        WHEN s.spread_efectivo = 0 THEN NULL
+        ELSE c.costo_fondos / s.spread_efectivo
+    END AS proporcion_del_spread_destinada_a_cubrir_costo_fondos,
+    CASE
+        WHEN s.spread_efectivo = 0 THEN NULL
+        ELSE (c.costo_fondos / s.spread_efectivo) * 100
+    END AS porcentaje_del_spread_destinado_a_cubrir_costo_fondos
+FROM spread s
+JOIN costo c
+  ON s."Año" = c."Año"
+ORDER BY s."Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Indicador %" AS "Costo Promedio de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Saldo Bs" AS monto_disponibilidades_bs
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Disponible en Bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto depositado en bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT
+  t_total."Año",
+  t_total."Trimestre",
+  t_vencida."cartera_vencida_bs",
+  t_total."cartera_total_bs",
+  ROUND((t_vencida."cartera_vencida_bs" / NULLIF(t_total."cartera_total_bs", 0)) * 100, 2) AS "porcentaje_cartera_vencida"
+FROM (
+  SELECT
+    "Año",
+    "Trimestre",
+    SUM("Monto Bs") AS "cartera_total_bs"
+  FROM "S_BOASFI66_000728"
+  WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+    AND "Trimestre" = 'IV'
+    AND "Entidad" = 'BNA'
+    AND "Tipo Crédito" = 'Crédito de Consumo'
+  GROUP BY "Año", "Trimestre"
+) t_total
+JOIN (
+  SELECT
+    "Año",
+    "Trimestre",
+    SUM("Monto Bs") AS "cartera_vencida_bs"
+  FROM "S_BOASFI66_000728"
+  WHERE "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+    AND "Trimestre" = 'IV'
+    AND "Entidad" = 'BNA'
+    AND "Tipo Crédito" = 'Crédito de Consumo'
+    AND "Estado Cartera" = 'Vencida'
+  GROUP BY "Año", "Trimestre"
+) t_vencida
+  ON t_total."Año" = t_vencida."Año"
+ AND t_total."Trimestre" = t_vencida."Trimestre";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Indicador %"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX(CASE
+    WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %"
+  END) AS "spread_efectivo",
+  MAX(CASE
+    WHEN "Indicador Nv2" = '   Costo Promedio de Fondos' THEN "Indicador %"
+  END) AS "costo_promedio_fondos",
+  CASE
+    WHEN MAX(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END) = 0 THEN NULL
+    ELSE MAX(CASE WHEN "Indicador Nv2" = '   Costo Promedio de Fondos' THEN "Indicador %" END)
+         / MAX(CASE WHEN "Indicador Nv2" = 'SPREAD EFECTIVO' THEN "Indicador %" END)
+  END AS "proporcion_del_spread_usada_para_cubrir_fondos"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND "Indicador Nv2" IN ('SPREAD EFECTIVO', '   Costo Promedio de Fondos')
+GROUP BY "Año"</t>
+  </si>
+  <si>
+    <t>Parece que no se han encontrado tablas válidas para obtener el "costo de los fondos" del Banco de Crédito (BCR) para los años 2024 y 2025. Todas las tablas candidatas incumplen con los requisitos necesarios:
+SPIM_50013_IF: No cumple con los filtros necesarios. Falta información sobre el costo de los fondos para los años 2024 y 2025 en un indicador financiero mensual.
+S_BOFINR44_00387: También incumple con los filtros requeridos. No incluye el costo de los fondos específico para el BCR en los años indicados.
+S_BOSBEF44_000392: Falta información sobre el costo de los fondos y no es válida para los indicadores financieros mensuales solicitados.
+Puedo intentar buscar nuevamente o explorar alternativas para obtener la información requerida. ¿Te gustaría que haga eso?</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Mes" = 'Diciembre'
+  AND "Entidad Financiera" = 'BIS'
+  AND "Cuenta Nv1" = '100.00 ACTIVO'
+  AND "Cuenta Nv3" = '113.00 BANCOS Y CORRESPONSALES DEL PAÍS'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Saldo Bs" AS "Monto Disponibilidades Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Tipo Entidad Financiera" = 'Banco'
+  AND "Cuenta Nv2" = '110.00 DISPONIBILIDADES'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "Activo Disponible Cierre Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "Monto Disponible en Bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Monto Acumulado Bs") AS "monto_depositado_bancos_bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Cuenta Financiera Nv4" = '1010201 Bancos'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año" DESC;</t>
+  </si>
+  <si>
+    <t>SELECT
+  t."Año",
+  t."Entidad",
+  SUM(CASE
+        WHEN t."Estado Cartera" IN ('Vencida', 'Reprogramada o reestructurada vencida')
+        THEN t."Monto Bs"
+        ELSE 0
+      END) AS "cartera_vencida_bs",
+  SUM(CASE
+        WHEN t."Estado Cartera" IN ('Vigente', 'Vencida', 'Reprogramada o reestructurada vigente', 'Reprogramada o reestructurada vencida', 'Contingente')
+        THEN t."Monto Bs"
+        ELSE 0
+      END) AS "cartera_total_bs",
+  CASE
+    WHEN SUM(CASE
+               WHEN t."Estado Cartera" IN ('Vigente', 'Vencida', 'Reprogramada o reestructurada vigente', 'Reprogramada o reestructurada vencida', 'Contingente')
+               THEN t."Monto Bs"
+               ELSE 0
+             END) = 0 THEN NULL
+    ELSE SUM(CASE
+               WHEN t."Estado Cartera" IN ('Vencida', 'Reprogramada o reestructurada vencida')
+               THEN t."Monto Bs"
+               ELSE 0
+             END)
+         / SUM(CASE
+                 WHEN t."Estado Cartera" IN ('Vigente', 'Vencida', 'Reprogramada o reestructurada vigente', 'Reprogramada o reestructurada vencida', 'Contingente')
+                 THEN t."Monto Bs"
+                 ELSE 0
+               END)
+  END AS "ratio_cartera_vencida_sobre_total"
+FROM "S_BOASFI66_000728" t
+WHERE t."Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+  AND t."Trimestre" = 'IV'
+  AND t."Entidad" = 'BNA'
+  AND t."Tipo Crédito" IN (
+    'Crédito de Consumo',
+    'Crédito de Consumo Garantizado con Garantía Real',
+    'Crédito de Consumo debidamente Garantizado'
+  )
+  AND t."Estado Cartera" IN (
+    'Vigente',
+    'Vencida',
+    'Reprogramada o reestructurada vigente',
+    'Reprogramada o reestructurada vencida',
+    'Contingente'
+  )
+GROUP BY t."Año", t."Entidad";</t>
+  </si>
+  <si>
+    <t>SELECT "Año", AVG("Indicador %") AS "Costo Promedio de Fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Tipo Entidad" = 'Banco'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  se."Año",
+  MAX(CASE
+    WHEN se."Indicador Nv1" = 'CÁLCULO SPREAD EFECTIVO'
+     AND se."Indicador Nv2" = 'CÁLCULO SPREAD EFECTIVO - SPREAD EFECTIVO'
+    THEN se."Indicador %"
+  END) AS "spread_efectivo_pct",
+  MAX(CASE
+    WHEN cpf."Indicador Nv2" = '   Costo Promedio de Fondos'
+    THEN cpf."Indicador %"
+  END) AS "costo_fondos_pct",
+  CASE
+    WHEN MAX(CASE WHEN se."Indicador Nv1" = 'CÁLCULO SPREAD EFECTIVO'
+                   AND se."Indicador Nv2" = 'CÁLCULO SPREAD EFECTIVO - SPREAD EFECTIVO'
+              THEN se."Indicador %" END) = 0
+    THEN NULL
+    ELSE
+      MAX(CASE WHEN cpf."Indicador Nv2" = '   Costo Promedio de Fondos'
+           THEN cpf."Indicador %" END)
+      / MAX(CASE WHEN se."Indicador Nv1" = 'CÁLCULO SPREAD EFECTIVO'
+                  AND se."Indicador Nv2" = 'CÁLCULO SPREAD EFECTIVO - SPREAD EFECTIVO'
+             THEN se."Indicador %" END)
+  END AS "proporcion_spread_destinada_a_costo_fondos"
+FROM "SPIM_50013_IF" se
+JOIN "SPIM_50013_IF" cpf
+  ON se."Entidad Financiera" = cpf."Entidad Financiera"
+ AND se."Año" = cpf."Año"
+ AND se."Mes" = cpf."Mes"
+WHERE se."Entidad Financiera" = 'CCB'
+  AND cpf."Entidad Financiera" = 'CCB'
+  AND se."Tipo Entidad" = 'Banco'
+  AND cpf."Tipo Entidad" = 'Banco'
+  AND se."Indicador Nv2" = 'SPREAD EFECTIVO'
+  AND cpf."Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND se."Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND cpf."Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND se."Mes" = 'Diciembre'
+  AND cpf."Mes" = 'Diciembre'
+GROUP BY se."Año"
+ORDER BY se."Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  "Entidad Financiera",
+  "Indicador Nv2",
+  "Mes",
+  "Indicador %" AS "Costo Promedio de Fondos %"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Tipo Entidad" = 'Banco'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Saldo Bs") AS "Monto Activo Disponible Bs"
+FROM "S_BOSBEF44_000392"
+WHERE "Entidad Financiera" = 'BIS'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOSBEF44_000392") - 3
+  AND "Cuenta Nv1" = '100.00 ACTIVO'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Disponible Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA'
+  AND "Cuenta Financiera Nv1" = '1 ACTIVO'
+  AND "Cuenta Financiera Nv2" = '101 DISPONIBLE'
+  AND "Cuenta Financiera Nv3" = '10102 BANCOS Y ENTIDADES FINANCIERAS'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  SUM("Monto Acumulado Bs") AS "Monto Depositado en Bancos Bs"
+FROM "S_BOAPS_44_000612"
+WHERE "Aseguradora" = 'BISA Seguros'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "S_BOAPS_44_000612") - 3
+  AND "Cuenta Financiera Nv1" = '7 CUENTAS DE ORDEN ACREEDORAS'
+  AND "Cuenta Financiera Nv2" = '702 DOCUMENTOS RECIBIDOS EN CUSTODIA'
+  AND "Cuenta Financiera Nv3" = '70201 DEPOSITADOS EN LA ENTIDAD'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>WITH cartera_consumo AS (
+    SELECT
+        "Año",
+        SUM(CASE WHEN "Estado Cartera" IN ('Vencida', 'Reprogramada o reestructurada vencida') THEN "Monto Bs" ELSE 0 END) AS cartera_vencida_bs,
+        SUM(CASE WHEN "Estado Cartera" IN ('Vigente', 'Reprogramada o reestructurada vigente', 'Vencida', 'Reprogramada o reestructurada vencida') THEN "Monto Bs" ELSE 0 END) AS cartera_total_bs
+    FROM "S_BOASFI66_000728"
+    WHERE "Entidad" = 'BNA'
+      AND "Tipo Crédito" = 'Crédito de Consumo'
+      AND "Trimestre" = 'IV'
+      AND "Año" = (SELECT MAX("Año") FROM "S_BOASFI66_000728")
+    GROUP BY "Año"
+), garantia_depositos AS (
+    SELECT
+        "Año",
+        SUM("Monto Bs") AS cartera_garantia_depositos_bs
+    FROM "clf_crt_tip_gar"
+    WHERE "Entidad" = 'BNA'
+      AND "Garantía Nv1" = 'Depositos en la Entidad Financiera'
+      AND "Trimestre" = 'IV'
+      AND "Año" = (SELECT MAX("Año") FROM "clf_crt_tip_gar")
+    GROUP BY "Año"
+)
+SELECT
+    c."Año",
+    c.cartera_vencida_bs,
+    c.cartera_total_bs,
+    g.cartera_garantia_depositos_bs
+FROM cartera_consumo c
+LEFT JOIN garantia_depositos g
+    ON c."Año" = g."Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  AVG("Indicador %") AS "Costo de los fondos"
+FROM "SPIM_50013_IF"
+WHERE "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Entidad Financiera" = 'BCR'
+  AND "Mes" = 'Diciembre'
+  AND "Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  se."Año",
+  MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END) AS "spread_efectivo_pct",
+  MAX(CASE WHEN se."Indicador Nv2" = '   Costo Promedio de Fondos' THEN se."Indicador %" END) AS "costo_promedio_fondos_pct",
+  CASE
+    WHEN MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END) = 0 THEN NULL
+    ELSE MAX(CASE WHEN se."Indicador Nv2" = '   Costo Promedio de Fondos' THEN se."Indicador %" END)
+         / MAX(CASE WHEN se."Indicador Nv2" = 'SPREAD EFECTIVO' THEN se."Indicador %" END)
+  END AS "proporcion_del_spread_destinada_a_cubrir_costo_fondos"
+FROM "SPIM_50013_IF" se
+WHERE se."Entidad Financiera" = 'BCR'
+  AND se."Indicador Nv2" IN ('SPREAD EFECTIVO', '   Costo Promedio de Fondos')
+  AND se."Año" &gt; (SELECT MAX("Año") FROM "SPIM_50013_IF") - 2
+  AND se."Mes" = 'Diciembre'
+GROUP BY se."Año"
+ORDER BY se."Año";</t>
+  </si>
+  <si>
+    <t>SELECT
+  "Año",
+  MAX("Indicador %") AS "Costo de fondos (%)"
+FROM "SPIM_50013_IF"
+WHERE "Entidad Financiera" = 'BCR'
+  AND "Indicador Nv2" = '   Costo Promedio de Fondos'
+  AND "Año" IN (2024, 2025)
+  AND "Mes" = 'Diciembre'
+GROUP BY "Año"
+ORDER BY "Año";</t>
+  </si>
 </sst>
 </file>
 
@@ -1740,7 +2478,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1750,6 +2488,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1766,13 +2510,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2192,17 +2937,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA3DAC64-27D9-415F-8378-E358F31B9411}">
   <dimension ref="A1:M11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="80.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="80.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="13" width="80.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="80.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="80.90625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="13" width="80.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2243,7 +2988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -2284,7 +3029,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>26</v>
       </c>
@@ -2325,7 +3070,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -2366,7 +3111,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -2407,7 +3152,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="230.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="232" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -2448,7 +3193,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>61</v>
       </c>
@@ -2489,7 +3234,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>67</v>
       </c>
@@ -2530,7 +3275,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>71</v>
       </c>
@@ -2571,7 +3316,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>76</v>
       </c>
@@ -2612,7 +3357,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>85</v>
       </c>
@@ -2664,13 +3409,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EC7178C-3D88-4FA7-9D2E-D58220DB2055}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="109.6640625" customWidth="1"/>
-    <col min="4" max="4" width="60.88671875" customWidth="1"/>
+    <col min="1" max="1" width="109.6328125" customWidth="1"/>
+    <col min="4" max="4" width="60.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -2681,7 +3426,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2695,7 +3440,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -2712,7 +3457,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -2729,7 +3474,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -2740,7 +3485,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>106</v>
       </c>
@@ -2751,7 +3496,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>108</v>
       </c>
@@ -2759,7 +3504,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>110</v>
       </c>
@@ -2767,7 +3512,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>112</v>
       </c>
@@ -2775,7 +3520,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>114</v>
       </c>
@@ -2784,7 +3529,7 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>117</v>
       </c>
@@ -2800,9 +3545,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38F382CB-3264-4364-8BC0-86B6B1186798}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -2819,7 +3564,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2830,7 +3575,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -2841,7 +3586,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -2855,7 +3600,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>106</v>
       </c>
@@ -2869,7 +3614,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>108</v>
       </c>
@@ -2883,7 +3628,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -2897,7 +3642,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -2911,7 +3656,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>114</v>
       </c>
@@ -2925,7 +3670,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -2947,9 +3692,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72D89B5-A94F-4B95-9307-F1034D484F2C}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>118</v>
       </c>
@@ -2972,7 +3717,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2995,7 +3740,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -3018,7 +3763,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
@@ -3041,7 +3786,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>106</v>
       </c>
@@ -3061,7 +3806,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>108</v>
       </c>
@@ -3081,7 +3826,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>110</v>
       </c>
@@ -3101,7 +3846,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -3121,7 +3866,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>181</v>
       </c>
@@ -3141,7 +3886,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>139</v>
       </c>
@@ -3159,6 +3904,247 @@
       </c>
       <c r="G10" s="1" t="s">
         <v>184</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9EE99AD-7993-4585-880C-342DE66AE3F0}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C1" t="s">
+        <v>120</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="G1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="K8" s="2"/>
+    </row>
+    <row r="9" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>114</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>